<commit_message>
add the topic function
</commit_message>
<xml_diff>
--- a/fund_api.xlsx
+++ b/fund_api.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\lzfdd\backups\MyProjects\python_test\fundweb\JJBond\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20FBFA8B-72D1-4F87-B0AE-1AD1AEE2ACFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D432A900-507D-4E49-AFAE-6212DE177D33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{7068C037-8E11-473D-BF09-92FC6201B4E7}"/>
+    <workbookView xWindow="2352" yWindow="3768" windowWidth="17280" windowHeight="13236" xr2:uid="{7068C037-8E11-473D-BF09-92FC6201B4E7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="71">
   <si>
     <t>接口</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1623,6 +1623,127 @@
 });</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
+  <si>
+    <t>获取主题基金列表</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://api.fund.eastmoney.com/ZTJJ/GetBKRelTopicFundNew?callback=jQuery18306304851841656735_1776918973918&amp;sort=undefined&amp;sorttype=DESC&amp;pageindex=1&amp;pagesize=10&amp;tp=BK000096&amp;isbuy=1&amp;_=1776940130680</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>jQuery18306304851841656735_1776918973918({
+    "Data": [
+        {
+            "CORR_1Y": 69.0725,
+            "FCODE": "501008",
+            "RELATETYPE": "1",
+            "SYRQ": "2026-04-22",
+            "SOURCERATE": "0.00%",
+            "DWJZ": 0.9074,
+            "RZDF": 1.14,
+            "RATE": "0.00%",
+            "ISBUY": "1",
+            "MINSG": 10.0,
+            "SHORTNAME": "汇添富中证互联网医疗指数(LOF)C",
+            "SYL_Z": 1.43,
+            "SYL_Y": 0.99,
+            "SYL_3Y": -9.25,
+            "SYL_6Y": -1.47,
+            "SYL_1N": 1.52,
+            "SYL_2N": 12.37,
+            "SYL_3N": -18.94,
+            "SYL_JN": 0.31,
+            "SYL_LN": -9.26,
+            "ISSALES": "1",
+            "FTYPE": "指数型-股票",
+            "RELATION": 69.0725
+        },
+        {
+            "CORR_1Y": 69.0725,
+            "FCODE": "501007",
+            "RELATETYPE": "1",
+            "SYRQ": "2026-04-22",
+            "SOURCERATE": "0.80%",
+            "DWJZ": 0.9375,
+            "RZDF": 1.13,
+            "RATE": "0.08%",
+            "ISBUY": "1",
+            "MINSG": 10.0,
+            "SHORTNAME": "汇添富中证互联网医疗指数(LOF)A",
+            "SYL_Z": 1.44,
+            "SYL_Y": 1.02,
+            "SYL_3Y": -9.17,
+            "SYL_6Y": -1.27,
+            "SYL_1N": 1.94,
+            "SYL_2N": 13.27,
+            "SYL_3N": -17.96,
+            "SYL_JN": 0.43,
+            "SYL_LN": -6.25,
+            "ISSALES": "1",
+            "FTYPE": "指数型-股票",
+            "RELATION": 69.0725
+        },
+    ],
+    "ErrCode": 0,
+    "ErrMsg": null,
+    "TotalCount": 62,
+    "Expansion": null,
+    "PageSize": 10,
+    "PageIndex": 1
+})</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>tp参数从 获取行业板块涨跌情况接口获取</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>获取板块主题详情</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://api.fund.eastmoney.com/ZTJJ/GetBKDetailInfoNew?callback=jQuery18306304851841656735_1776918973918&amp;tp=BK000197&amp;_=1776943829756</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>jQuery18306304851841656735_1776918973918({
+    "Data": {
+        "M": -4.0300,
+        "MSC": 184.0,
+        "Q": 17.2200,
+        "QSC": 184.0,
+        "RANKM": 183.0,
+        "RANKQ": 17.0,
+        "RANKSY": 56.0,
+        "RANKW": 63.0,
+        "RANKY": 98.0,
+        "SEC_CODE": "BK000197",
+        "SEC_NAME": "能源",
+        "SYSC": 184.0,
+        "W": 2.0100,
+        "WSC": 185.0,
+        "Y": 44.9200,
+        "YSC": 184.0,
+        "INDEXNAME": "能源",
+        "INDEXCODE": "BK000197",
+        "D": 2.785084,
+        "SY": 17.2300
+    },
+    "ErrCode": 0,
+    "ErrMsg": null,
+    "TotalCount": 0,
+    "Expansion": null,
+    "PageSize": 0,
+    "PageIndex": 0
+})</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>响应参数中，"D"为日涨幅，"W" 为近一周涨幅，"M"为近一月，"Q"为近三月，"Y"为近一年，“SY”为今年来涨幅。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -2014,7 +2135,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{756FAFE1-58E3-4702-9EE8-9320214AB644}">
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="1"/>
@@ -2284,6 +2405,34 @@
         <v>62</v>
       </c>
     </row>
+    <row r="17" spans="2:7" ht="409.6" x14ac:dyDescent="0.25">
+      <c r="B17" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" ht="409.6" x14ac:dyDescent="0.25">
+      <c r="B18" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
@@ -2297,6 +2446,7 @@
     <hyperlink ref="C11" r:id="rId8" display="https://push2.eastmoney.com/api/qt/stock/trends2/get?fields1=f1,f2,f3,f4,f5,f6,f7,f8,f9,f10,f11,f12,f13,f14,f17&amp;fields2=f51,f52,f53,f54,f55,f58&amp;dect=1&amp;mpi=1000&amp;ut=bd1d9ddb04089700cf9c27f6f7426281&amp;secid=100.DJIA&amp;ndays=1&amp;iscr=0&amp;iscca=0&amp;wbp2u=1849325530509956|0|1|0|web&amp;cb=miniquotechart_jp152" xr:uid="{18F47342-9A41-47AC-A7DD-1F5487D4AEB2}"/>
     <hyperlink ref="C13" r:id="rId9" display="https://push2.eastmoney.com/api/qt/stock/trends2/get?fields1=f1,f2,f3,f4,f5,f6,f7,f8,f9,f10,f11,f12,f13,f14,f17&amp;fields2=f51,f52,f53,f54,f55,f58&amp;dect=1&amp;mpi=1000&amp;ut=bd1d9ddb04089700cf9c27f6f7426281&amp;secid=100.HSCEI&amp;ndays=1&amp;iscr=0&amp;iscca=0&amp;wbp2u=1849325530509956|0|1|0|web&amp;cb=miniquotechart_jp248" xr:uid="{36FC8E56-4897-4C0B-A7F3-540876EE494B}"/>
     <hyperlink ref="C14" r:id="rId10" display="https://push2.eastmoney.com/api/qt/stock/trends2/get?fields1=f1,f2,f3,f4,f5,f6,f7,f8,f9,f10,f11,f12,f13,f14,f17&amp;fields2=f51,f52,f53,f54,f55,f58&amp;dect=1&amp;mpi=1000&amp;ut=bd1d9ddb04089700cf9c27f6f7426281&amp;secid=124.HSCCI&amp;ndays=1&amp;iscr=0&amp;iscca=0&amp;wbp2u=1849325530509956|0|1|0|web&amp;cb=miniquotechart_jp250" xr:uid="{F0EC10B8-513A-4B2E-A66E-991476046EFD}"/>
+    <hyperlink ref="C17" r:id="rId11" xr:uid="{A628F64C-A7D6-4A1F-89ED-5FBC668A5C95}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>